<commit_message>
multitask-ssl-rotation: add per-model perf plots + refresh results workbook
plot_perf_by_model.py renders per-model performance bars for classification, regression, and static-LP; build_results_xlsx.py and the results xlsx refreshed to match.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/experiments/multitask_ssl_rotation/multitask_ssl_rotation_results.xlsx
+++ b/scripts/experiments/multitask_ssl_rotation/multitask_ssl_rotation_results.xlsx
@@ -9,12 +9,14 @@
   <sheets>
     <sheet name="About" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Summary_T1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Classification" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Regression" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Static_link_prediction" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Raw_classification" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Raw_regression" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Raw_static_link_prediction" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Overall_ranking" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Classification" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Regression" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Regression_ranks" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Static_link_prediction" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Raw_classification" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Raw_regression" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Raw_static_link_prediction" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +30,7 @@
     <numFmt numFmtId="165" formatCode="+0.000;\-0.000;0.000"/>
     <numFmt numFmtId="166" formatCode="0.0000####"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,6 +66,18 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="5">
@@ -115,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -154,13 +168,44 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -280,6 +325,61 @@
 </file>
 
 <file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>results</author>
+  </authors>
+  <commentList>
+    <comment ref="E4" authorId="0" shapeId="0">
+      <text>
+        <t>= mean of the 3 target ranks to the left (each target rank is itself a mean over 4 graphs — see Regression_ranks).</t>
+      </text>
+    </comment>
+    <comment ref="H4" authorId="0" shapeId="0">
+      <text>
+        <t>= mean of the 2 per-graph ranks to the left.</t>
+      </text>
+    </comment>
+    <comment ref="M4" authorId="0" shapeId="0">
+      <text>
+        <t>= mean of the 4 per-graph ranks to the left.</t>
+      </text>
+    </comment>
+    <comment ref="N4" authorId="0" shapeId="0">
+      <text>
+        <t>Equal-weight mean of Reg/Cls/sLP means — each task family counts once, so regression's 12 instances don't outvote classification's 2.</t>
+      </text>
+    </comment>
+    <comment ref="O4" authorId="0" shapeId="0">
+      <text>
+        <t>max of the 3 task means: the family the model is weakest on. A generalist stays low; a collapsing specialist hits 4.</t>
+      </text>
+    </comment>
+    <comment ref="P4" authorId="0" shapeId="0">
+      <text>
+        <t>(4 - OVERALL rank)/3. 1.00 = always ranked best of 4; 0.00 = always worst.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>results</author>
+  </authors>
+  <commentList>
+    <comment ref="E4" authorId="0" shapeId="0">
+      <text>
+        <t>Mean rank over all 12 target×dataset instances. 1 = always best of the 4 models, 4 = always worst.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>results</author>
@@ -879,6 +979,756 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>shots</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>roc_auc</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>f1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>midterm</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="9" t="inlineStr"/>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>eval_CL_to_midterm_slp_0shot_09_07_2026_17_28_00</t>
+        </is>
+      </c>
+      <c r="H2" s="32" t="n">
+        <v>0.416752375</v>
+      </c>
+      <c r="I2" s="32" t="n">
+        <v>0.498</v>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>0.664886515353805</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>midterm</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="9" t="inlineStr"/>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>eval_FP_to_midterm_slp_0shot_09_07_2026_17_28_00</t>
+        </is>
+      </c>
+      <c r="H3" s="32" t="n">
+        <v>0.433355</v>
+      </c>
+      <c r="I3" s="32" t="n">
+        <v>0.5465</v>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>0.6625744047619048</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>midterm</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="9" t="inlineStr"/>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>eval_NM_to_midterm_slp_0shot_09_07_2026_17_28_00</t>
+        </is>
+      </c>
+      <c r="H4" s="32" t="n">
+        <v>0.48701</v>
+      </c>
+      <c r="I4" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>MIX</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>midterm</t>
+        </is>
+      </c>
+      <c r="C5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="12" t="inlineStr"/>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G5" s="33" t="inlineStr">
+        <is>
+          <t>eval_MIX_to_midterm_slp_0shot_09_07_2026_17_28_01</t>
+        </is>
+      </c>
+      <c r="H5" s="34" t="n">
+        <v>0.676129875</v>
+      </c>
+      <c r="I5" s="34" t="n">
+        <v>0.64225</v>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>0.5343312723722746</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>ukr_rus_twitter</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr"/>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>eval_CL_to_ukr_rus_twitter_slp_0shot_09_07_2026_17_28_20</t>
+        </is>
+      </c>
+      <c r="H6" s="32" t="n">
+        <v>0.2875115</v>
+      </c>
+      <c r="I6" s="32" t="n">
+        <v>0.4995</v>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>0.6662220740246749</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>ukr_rus_twitter</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="9" t="inlineStr"/>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>eval_NM_to_ukr_rus_twitter_slp_0shot_09_07_2026_17_28_20</t>
+        </is>
+      </c>
+      <c r="H7" s="32" t="n">
+        <v>0.48371125</v>
+      </c>
+      <c r="I7" s="32" t="n">
+        <v>0.49975</v>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>ukr_rus_twitter</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="9" t="inlineStr"/>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>eval_FP_to_ukr_rus_twitter_slp_0shot_09_07_2026_17_28_21</t>
+        </is>
+      </c>
+      <c r="H8" s="32" t="n">
+        <v>0.53384625</v>
+      </c>
+      <c r="I8" s="32" t="n">
+        <v>0.55925</v>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>0.6713886300093197</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>MIX</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>ukr_rus_twitter</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="12" t="inlineStr"/>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G9" s="33" t="inlineStr">
+        <is>
+          <t>eval_MIX_to_ukr_rus_twitter_slp_0shot_09_07_2026_17_28_21</t>
+        </is>
+      </c>
+      <c r="H9" s="34" t="n">
+        <v>0.8612627499999999</v>
+      </c>
+      <c r="I9" s="34" t="n">
+        <v>0.779</v>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>0.7390791027154664</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>covid19_twitter</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr"/>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>eval_CL_to_covid19_twitter_slp_0shot_09_07_2026_17_34_22</t>
+        </is>
+      </c>
+      <c r="H10" s="32" t="n">
+        <v>0.366347875</v>
+      </c>
+      <c r="I10" s="32" t="n">
+        <v>0.49975</v>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>0.6661104622059069</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>covid19_twitter</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr"/>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>eval_FP_to_covid19_twitter_slp_0shot_09_07_2026_17_34_22</t>
+        </is>
+      </c>
+      <c r="H11" s="32" t="n">
+        <v>0.4486818750000001</v>
+      </c>
+      <c r="I11" s="32" t="n">
+        <v>0.52425</v>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>0.6356500095730423</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>covid19_twitter</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr"/>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>eval_NM_to_covid19_twitter_slp_0shot_09_07_2026_17_34_22</t>
+        </is>
+      </c>
+      <c r="H12" s="32" t="n">
+        <v>0.40565375</v>
+      </c>
+      <c r="I12" s="32" t="n">
+        <v>0.4995</v>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>MIX</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>covid19_twitter</t>
+        </is>
+      </c>
+      <c r="C13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="12" t="inlineStr"/>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G13" s="33" t="inlineStr">
+        <is>
+          <t>eval_MIX_to_covid19_twitter_slp_0shot_09_07_2026_17_34_25</t>
+        </is>
+      </c>
+      <c r="H13" s="34" t="n">
+        <v>0.75508</v>
+      </c>
+      <c r="I13" s="34" t="n">
+        <v>0.6765</v>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>0.5790500975927131</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>twibot20</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="9" t="inlineStr"/>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>eval_NM_to_twibot20_slp_0shot_09_07_2026_17_38_14</t>
+        </is>
+      </c>
+      <c r="H14" s="32" t="n">
+        <v>0.49065475</v>
+      </c>
+      <c r="I14" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>twibot20</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr"/>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>eval_CL_to_twibot20_slp_0shot_09_07_2026_17_38_17</t>
+        </is>
+      </c>
+      <c r="H15" s="32" t="n">
+        <v>0.2592245</v>
+      </c>
+      <c r="I15" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>0.6666666666666666</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>twibot20</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr"/>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>eval_FP_to_twibot20_slp_0shot_09_07_2026_17_38_17</t>
+        </is>
+      </c>
+      <c r="H16" s="32" t="n">
+        <v>0.381107125</v>
+      </c>
+      <c r="I16" s="32" t="n">
+        <v>0.5135</v>
+      </c>
+      <c r="J16" s="9" t="inlineStr">
+        <is>
+          <t>0.6497480201583873</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>MIX</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>twibot20</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="12" t="inlineStr"/>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>static_link_prediction</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G17" s="33" t="inlineStr">
+        <is>
+          <t>eval_MIX_to_twibot20_slp_0shot_09_07_2026_17_38_17</t>
+        </is>
+      </c>
+      <c r="H17" s="34" t="n">
+        <v>0.74460025</v>
+      </c>
+      <c r="I17" s="34" t="n">
+        <v>0.66475</v>
+      </c>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>0.566159818828858</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1127,6 +1977,413 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:P14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Overall model ranking — fair, cross-task, with full breakdown (lower rank = better)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Rank 1–4 per eval instance by the task's own metric (higher = better; ties averaged). Reg mean = mean of its 3 target ranks · Cls / sLP mean = mean of their per-graph ranks · OVERALL = equal-weight mean of the 3 task means.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Regression · rank by target</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="n"/>
+      <c r="D4" s="17" t="n"/>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>Reg mean</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>Classification · by graph</t>
+        </is>
+      </c>
+      <c r="G4" s="17" t="n"/>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
+          <t>Cls mean</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>Static-LP · rank by graph</t>
+        </is>
+      </c>
+      <c r="J4" s="17" t="n"/>
+      <c r="K4" s="17" t="n"/>
+      <c r="L4" s="17" t="n"/>
+      <c r="M4" s="16" t="inlineStr">
+        <is>
+          <t>sLP mean</t>
+        </is>
+      </c>
+      <c r="N4" s="16" t="inlineStr">
+        <is>
+          <t>OVERALL rank</t>
+        </is>
+      </c>
+      <c r="O4" s="16" t="inlineStr">
+        <is>
+          <t>Worst task</t>
+        </is>
+      </c>
+      <c r="P4" s="16" t="inlineStr">
+        <is>
+          <t>Score 0–1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="n"/>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>followers</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>statuses</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>account age</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="n"/>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>twibot20</t>
+        </is>
+      </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>election2020</t>
+        </is>
+      </c>
+      <c r="H5" s="17" t="n"/>
+      <c r="I5" s="18" t="inlineStr">
+        <is>
+          <t>midterm</t>
+        </is>
+      </c>
+      <c r="J5" s="18" t="inlineStr">
+        <is>
+          <t>ukr_rus</t>
+        </is>
+      </c>
+      <c r="K5" s="18" t="inlineStr">
+        <is>
+          <t>covid19</t>
+        </is>
+      </c>
+      <c r="L5" s="18" t="inlineStr">
+        <is>
+          <t>twibot20</t>
+        </is>
+      </c>
+      <c r="M5" s="17" t="n"/>
+      <c r="N5" s="17" t="n"/>
+      <c r="O5" s="17" t="n"/>
+      <c r="P5" s="17" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>MIX</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C6" s="20" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="D6" s="20" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>2.083333333333333</v>
+      </c>
+      <c r="F6" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" s="21" t="n">
+        <v>1.694444444444445</v>
+      </c>
+      <c r="O6" s="20" t="n">
+        <v>2.083333333333333</v>
+      </c>
+      <c r="P6" s="21" t="n">
+        <v>0.7685185185185185</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="24" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="F7" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="24" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I7" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K7" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="L7" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="M7" s="24" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N7" s="24" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="O7" s="23" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="P7" s="24" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="23" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="E8" s="24" t="n">
+        <v>1.333333333333333</v>
+      </c>
+      <c r="F8" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="I8" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="M8" s="24" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N8" s="24" t="n">
+        <v>2.611111111111111</v>
+      </c>
+      <c r="O8" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="P8" s="24" t="n">
+        <v>0.462962962962963</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="23" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E9" s="24" t="n">
+        <v>3.833333333333333</v>
+      </c>
+      <c r="F9" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="24" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I9" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="L9" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="M9" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" s="24" t="n">
+        <v>3.444444444444445</v>
+      </c>
+      <c r="O9" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="P9" s="24" t="n">
+        <v>0.1851851851851851</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>• Bold columns are aggregates; each equals the mean of the plain cells to its left — fully auditable in-place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>• Fair by construction: rank-based (Spearman ρ vs ROC-AUC scale is irrelevant) and each task family weighted equally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>• MIX is the best GENERAL model: lowest OVERALL rank AND lowest worst-task rank — the only arm that never drops to a family it can't do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>• FP wins regression outright but collapses to rank 4 on classification; NM is strong on cls/LP but ~rank 3 on regression; CL is last.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="M4:M5"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="I4:L4"/>
+    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="O4:O5"/>
+    <mergeCell ref="P4:P5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1179,7 +2436,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>twibot20</t>
         </is>
@@ -1198,7 +2455,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>election2020</t>
         </is>
@@ -1217,21 +2474,21 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>Mean</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="26" t="n">
         <v>0.8101052361111111</v>
       </c>
-      <c r="C7" s="18" t="n">
+      <c r="C7" s="26" t="n">
         <v>0.6377517708333333</v>
       </c>
-      <c r="D7" s="18" t="n">
+      <c r="D7" s="26" t="n">
         <v>0.4924334722222222</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="26" t="n">
         <v>0.7951280069444444</v>
       </c>
     </row>
@@ -1270,7 +2527,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>twibot20</t>
         </is>
@@ -1289,7 +2546,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>election2020</t>
         </is>
@@ -1312,7 +2569,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1370,7 +2627,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>midterm</t>
         </is>
@@ -1389,7 +2646,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>ukr_rus_twitter</t>
         </is>
@@ -1408,7 +2665,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>covid19_twitter</t>
         </is>
@@ -1427,7 +2684,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>twibot20 (held-out)</t>
         </is>
@@ -1446,21 +2703,21 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>Mean (all datasets × targets)</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n">
+      <c r="B9" s="26" t="n">
         <v>-0.0005497887857409633</v>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="26" t="n">
         <v>-0.1278291566439923</v>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="26" t="n">
         <v>0.1656251249080986</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="26" t="n">
         <v>0.09723651799777945</v>
       </c>
     </row>
@@ -1476,7 +2733,203 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Regression — general performance by mean rank (lower = better)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>On each (target × test-graph) instance the 4 models are ranked 1–4 by Spearman ρ; cells are mean ranks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>followers</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>statuses</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>account age</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>OVERALL rank</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Wins (rank-1, /12)</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Mean ρ (ref)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="E5" s="24" t="n">
+        <v>1.333333333333333</v>
+      </c>
+      <c r="F5" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>0.1656251249080986</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>MIX</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C6" s="20" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="D6" s="20" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>2.083333333333333</v>
+      </c>
+      <c r="F6" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" s="29" t="n">
+        <v>0.09723651799777945</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="24" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="F7" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>-0.0005497887857409633</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="23" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E8" s="24" t="n">
+        <v>3.833333333333333</v>
+      </c>
+      <c r="F8" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>-0.1278291566439923</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>• Mean rank = average finishing place (1–4) across the test graphs; lower is better. Range 1.00 (always best) to 4.00 (always worst).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>• FP is the regression specialist (best overall rank). MIX is 2nd overall and actually ranks best on account-age.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>• Wins = number of the 12 instances where the model has the single highest ρ. Mean ρ is the raw metric for reference (see Regression sheet).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1540,7 +2993,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>midterm</t>
         </is>
@@ -1562,7 +3015,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>ukr_rus_twitter</t>
         </is>
@@ -1584,7 +3037,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>covid19_twitter</t>
         </is>
@@ -1606,7 +3059,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>twibot20 (held-out)</t>
         </is>
@@ -1628,29 +3081,29 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>Mean</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n">
+      <c r="B9" s="26" t="n">
         <v>0.4667574375</v>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="26" t="n">
         <v>0.3324590625</v>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="26" t="n">
         <v>0.4492475625</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="26" t="n">
         <v>0.7592682187499999</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="30" t="n">
         <v>0.26922</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>MIX − max(control) per dataset: mean +0.269, range [+0.189, +0.327], all 4 positive.</t>
         </is>
@@ -1691,7 +3144,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>midterm</t>
         </is>
@@ -1710,7 +3163,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>ukr_rus_twitter</t>
         </is>
@@ -1729,7 +3182,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>covid19_twitter</t>
         </is>
@@ -1748,7 +3201,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>twibot20</t>
         </is>
@@ -1772,7 +3225,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1875,10 +3328,10 @@
           <t>eval_CL_to_twibot20_pl_10shot_09_07_2026_17_41_35</t>
         </is>
       </c>
-      <c r="H2" s="21" t="n">
+      <c r="H2" s="32" t="n">
         <v>0.6106375416666667</v>
       </c>
-      <c r="I2" s="21" t="n">
+      <c r="I2" s="32" t="n">
         <v>0.5836666666666667</v>
       </c>
       <c r="J2" s="9" t="inlineStr">
@@ -1917,10 +3370,10 @@
           <t>eval_FP_to_twibot20_pl_10shot_09_07_2026_17_41_36</t>
         </is>
       </c>
-      <c r="H3" s="21" t="n">
+      <c r="H3" s="32" t="n">
         <v>0.4895429444444445</v>
       </c>
-      <c r="I3" s="21" t="n">
+      <c r="I3" s="32" t="n">
         <v>0.5011666666666666</v>
       </c>
       <c r="J3" s="9" t="inlineStr">
@@ -1940,7 +3393,7 @@
           <t>twibot20</t>
         </is>
       </c>
-      <c r="C4" s="22" t="n">
+      <c r="C4" s="33" t="n">
         <v>10</v>
       </c>
       <c r="D4" s="12" t="inlineStr"/>
@@ -1954,15 +3407,15 @@
           <t>test</t>
         </is>
       </c>
-      <c r="G4" s="22" t="inlineStr">
+      <c r="G4" s="33" t="inlineStr">
         <is>
           <t>eval_MIX_to_twibot20_pl_10shot_09_07_2026_17_41_36</t>
         </is>
       </c>
-      <c r="H4" s="23" t="n">
+      <c r="H4" s="34" t="n">
         <v>0.6097460138888888</v>
       </c>
-      <c r="I4" s="23" t="n">
+      <c r="I4" s="34" t="n">
         <v>0.5839166666666666</v>
       </c>
       <c r="J4" s="12" t="inlineStr">
@@ -2001,10 +3454,10 @@
           <t>eval_NM_to_twibot20_pl_10shot_09_07_2026_17_41_36</t>
         </is>
       </c>
-      <c r="H5" s="21" t="n">
+      <c r="H5" s="32" t="n">
         <v>0.6398304722222221</v>
       </c>
-      <c r="I5" s="21" t="n">
+      <c r="I5" s="32" t="n">
         <v>0.5988333333333333</v>
       </c>
       <c r="J5" s="9" t="inlineStr">
@@ -2043,10 +3496,10 @@
           <t>eval_CL_to_election2020_pl_10shot_09_07_2026_17_41_53</t>
         </is>
       </c>
-      <c r="H6" s="21" t="n">
+      <c r="H6" s="32" t="n">
         <v>0.664866</v>
       </c>
-      <c r="I6" s="21" t="n">
+      <c r="I6" s="32" t="n">
         <v>0.639</v>
       </c>
       <c r="J6" s="9" t="inlineStr">
@@ -2085,10 +3538,10 @@
           <t>eval_NM_to_election2020_pl_10shot_09_07_2026_17_41_53</t>
         </is>
       </c>
-      <c r="H7" s="21" t="n">
+      <c r="H7" s="32" t="n">
         <v>0.98038</v>
       </c>
-      <c r="I7" s="21" t="n">
+      <c r="I7" s="32" t="n">
         <v>0.964</v>
       </c>
       <c r="J7" s="9" t="inlineStr">
@@ -2127,10 +3580,10 @@
           <t>eval_FP_to_election2020_pl_10shot_09_07_2026_17_41_54</t>
         </is>
       </c>
-      <c r="H8" s="21" t="n">
+      <c r="H8" s="32" t="n">
         <v>0.495324</v>
       </c>
-      <c r="I8" s="21" t="n">
+      <c r="I8" s="32" t="n">
         <v>0.5</v>
       </c>
       <c r="J8" s="9" t="inlineStr">
@@ -2150,7 +3603,7 @@
           <t>election2020</t>
         </is>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C9" s="33" t="n">
         <v>10</v>
       </c>
       <c r="D9" s="12" t="inlineStr"/>
@@ -2164,15 +3617,15 @@
           <t>test</t>
         </is>
       </c>
-      <c r="G9" s="22" t="inlineStr">
+      <c r="G9" s="33" t="inlineStr">
         <is>
           <t>eval_MIX_to_election2020_pl_10shot_09_07_2026_17_41_54</t>
         </is>
       </c>
-      <c r="H9" s="23" t="n">
+      <c r="H9" s="34" t="n">
         <v>0.98051</v>
       </c>
-      <c r="I9" s="23" t="n">
+      <c r="I9" s="34" t="n">
         <v>0.968</v>
       </c>
       <c r="J9" s="12" t="inlineStr">
@@ -2186,7 +3639,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2305,16 +3758,16 @@
           <t>eval_NM_to_midterm_reg_10shot_statuses_count_09_07_2026_17_05_36</t>
         </is>
       </c>
-      <c r="H2" s="21" t="n">
+      <c r="H2" s="32" t="n">
         <v>-0.01571106728160299</v>
       </c>
-      <c r="I2" s="21" t="n">
+      <c r="I2" s="32" t="n">
         <v>9.600422977030263</v>
       </c>
-      <c r="J2" s="21" t="n">
+      <c r="J2" s="32" t="n">
         <v>9.402083396911621</v>
       </c>
-      <c r="K2" s="21" t="n">
+      <c r="K2" s="32" t="n">
         <v>-23.85382652282715</v>
       </c>
       <c r="L2" s="9" t="inlineStr">
@@ -2357,16 +3810,16 @@
           <t>eval_CL_to_midterm_reg_10shot_followers_count_09_07_2026_17_05_36</t>
         </is>
       </c>
-      <c r="H3" s="21" t="n">
+      <c r="H3" s="32" t="n">
         <v>-0.2087703890274008</v>
       </c>
-      <c r="I3" s="21" t="n">
+      <c r="I3" s="32" t="n">
         <v>6.433892285404345</v>
       </c>
-      <c r="J3" s="21" t="n">
+      <c r="J3" s="32" t="n">
         <v>6.050000190734863</v>
       </c>
-      <c r="K3" s="21" t="n">
+      <c r="K3" s="32" t="n">
         <v>-8.122678756713867</v>
       </c>
       <c r="L3" s="9" t="inlineStr">
@@ -2409,16 +3862,16 @@
           <t>eval_NM_to_midterm_reg_10shot_followers_count_09_07_2026_17_05_36</t>
         </is>
       </c>
-      <c r="H4" s="21" t="n">
+      <c r="H4" s="32" t="n">
         <v>-0.05553915039591011</v>
       </c>
-      <c r="I4" s="21" t="n">
+      <c r="I4" s="32" t="n">
         <v>6.36659254793227</v>
       </c>
-      <c r="J4" s="21" t="n">
+      <c r="J4" s="32" t="n">
         <v>5.992841243743896</v>
       </c>
-      <c r="K4" s="21" t="n">
+      <c r="K4" s="32" t="n">
         <v>-7.932826995849609</v>
       </c>
       <c r="L4" s="9" t="inlineStr">
@@ -2461,16 +3914,16 @@
           <t>eval_NM_to_midterm_reg_10shot_account_age_days_09_07_2026_17_05_36</t>
         </is>
       </c>
-      <c r="H5" s="21" t="n">
+      <c r="H5" s="32" t="n">
         <v>-0.06132001602827829</v>
       </c>
-      <c r="I5" s="21" t="n">
+      <c r="I5" s="32" t="n">
         <v>7.466696229376625</v>
       </c>
-      <c r="J5" s="21" t="n">
+      <c r="J5" s="32" t="n">
         <v>7.347213745117188</v>
       </c>
-      <c r="K5" s="21" t="n">
+      <c r="K5" s="32" t="n">
         <v>-32.038818359375</v>
       </c>
       <c r="L5" s="9" t="inlineStr">
@@ -2513,16 +3966,16 @@
           <t>eval_FP_to_midterm_reg_10shot_followers_count_09_07_2026_17_05_52</t>
         </is>
       </c>
-      <c r="H6" s="21" t="n">
+      <c r="H6" s="32" t="n">
         <v>0.2846323982472672</v>
       </c>
-      <c r="I6" s="21" t="n">
+      <c r="I6" s="32" t="n">
         <v>6.144469787717079</v>
       </c>
-      <c r="J6" s="21" t="n">
+      <c r="J6" s="32" t="n">
         <v>5.770872592926025</v>
       </c>
-      <c r="K6" s="21" t="n">
+      <c r="K6" s="32" t="n">
         <v>-7.320389747619629</v>
       </c>
       <c r="L6" s="9" t="inlineStr">
@@ -2565,16 +4018,16 @@
           <t>eval_CL_to_midterm_reg_10shot_account_age_days_09_07_2026_17_05_52</t>
         </is>
       </c>
-      <c r="H7" s="21" t="n">
+      <c r="H7" s="32" t="n">
         <v>-0.04165117141385686</v>
       </c>
-      <c r="I7" s="21" t="n">
+      <c r="I7" s="32" t="n">
         <v>7.531098803510178</v>
       </c>
-      <c r="J7" s="21" t="n">
+      <c r="J7" s="32" t="n">
         <v>7.41242504119873</v>
       </c>
-      <c r="K7" s="21" t="n">
+      <c r="K7" s="32" t="n">
         <v>-32.61121368408203</v>
       </c>
       <c r="L7" s="9" t="inlineStr">
@@ -2617,16 +4070,16 @@
           <t>eval_CL_to_midterm_reg_10shot_statuses_count_09_07_2026_17_05_52</t>
         </is>
       </c>
-      <c r="H8" s="21" t="n">
+      <c r="H8" s="32" t="n">
         <v>-0.2189998601886188</v>
       </c>
-      <c r="I8" s="21" t="n">
+      <c r="I8" s="32" t="n">
         <v>9.680657708389042</v>
       </c>
-      <c r="J8" s="21" t="n">
+      <c r="J8" s="32" t="n">
         <v>9.473175048828125</v>
       </c>
-      <c r="K8" s="21" t="n">
+      <c r="K8" s="32" t="n">
         <v>-24.27098846435547</v>
       </c>
       <c r="L8" s="9" t="inlineStr">
@@ -2669,16 +4122,16 @@
           <t>eval_FP_to_midterm_reg_10shot_statuses_count_09_07_2026_17_05_52</t>
         </is>
       </c>
-      <c r="H9" s="21" t="n">
+      <c r="H9" s="32" t="n">
         <v>0.2095705790198308</v>
       </c>
-      <c r="I9" s="21" t="n">
+      <c r="I9" s="32" t="n">
         <v>9.379758313934962</v>
       </c>
-      <c r="J9" s="21" t="n">
+      <c r="J9" s="32" t="n">
         <v>9.182087898254395</v>
       </c>
-      <c r="K9" s="21" t="n">
+      <c r="K9" s="32" t="n">
         <v>-22.72443008422852</v>
       </c>
       <c r="L9" s="9" t="inlineStr">
@@ -2698,7 +4151,7 @@
           <t>midterm</t>
         </is>
       </c>
-      <c r="C10" s="22" t="n">
+      <c r="C10" s="33" t="n">
         <v>10</v>
       </c>
       <c r="D10" s="12" t="inlineStr">
@@ -2716,21 +4169,21 @@
           <t>test</t>
         </is>
       </c>
-      <c r="G10" s="22" t="inlineStr">
+      <c r="G10" s="33" t="inlineStr">
         <is>
           <t>eval_MIX_to_midterm_reg_10shot_account_age_days_09_07_2026_17_06_10</t>
         </is>
       </c>
-      <c r="H10" s="23" t="n">
+      <c r="H10" s="34" t="n">
         <v>0.1530965379995686</v>
       </c>
-      <c r="I10" s="23" t="n">
+      <c r="I10" s="34" t="n">
         <v>7.195775053417441</v>
       </c>
-      <c r="J10" s="23" t="n">
+      <c r="J10" s="34" t="n">
         <v>7.080020904541016</v>
       </c>
-      <c r="K10" s="23" t="n">
+      <c r="K10" s="34" t="n">
         <v>-29.68475532531738</v>
       </c>
       <c r="L10" s="12" t="inlineStr">
@@ -2750,7 +4203,7 @@
           <t>midterm</t>
         </is>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="33" t="n">
         <v>10</v>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -2768,21 +4221,21 @@
           <t>test</t>
         </is>
       </c>
-      <c r="G11" s="22" t="inlineStr">
+      <c r="G11" s="33" t="inlineStr">
         <is>
           <t>eval_MIX_to_midterm_reg_10shot_followers_count_09_07_2026_17_06_10</t>
         </is>
       </c>
-      <c r="H11" s="23" t="n">
+      <c r="H11" s="34" t="n">
         <v>0.2343851458574698</v>
       </c>
-      <c r="I11" s="23" t="n">
+      <c r="I11" s="34" t="n">
         <v>6.106245014731364</v>
       </c>
-      <c r="J11" s="23" t="n">
+      <c r="J11" s="34" t="n">
         <v>5.737428188323975</v>
       </c>
-      <c r="K11" s="23" t="n">
+      <c r="K11" s="34" t="n">
         <v>-7.217188835144043</v>
       </c>
       <c r="L11" s="12" t="inlineStr">
@@ -2802,7 +4255,7 @@
           <t>midterm</t>
         </is>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="33" t="n">
         <v>10</v>
       </c>
       <c r="D12" s="12" t="inlineStr">
@@ -2820,21 +4273,21 @@
           <t>test</t>
         </is>
       </c>
-      <c r="G12" s="22" t="inlineStr">
+      <c r="G12" s="33" t="inlineStr">
         <is>
           <t>eval_MIX_to_midterm_reg_10shot_statuses_count_09_07_2026_17_06_10</t>
         </is>
       </c>
-      <c r="H12" s="23" t="n">
+      <c r="H12" s="34" t="n">
         <v>0.1452252005039579</v>
       </c>
-      <c r="I12" s="23" t="n">
+      <c r="I12" s="34" t="n">
         <v>9.319176655039437</v>
       </c>
-      <c r="J12" s="23" t="n">
+      <c r="J12" s="34" t="n">
         <v>9.122258186340332</v>
       </c>
-      <c r="K12" s="23" t="n">
+      <c r="K12" s="34" t="n">
         <v>-22.41895866394043</v>
       </c>
       <c r="L12" s="12" t="inlineStr">
@@ -2877,16 +4330,16 @@
           <t>eval_FP_to_midterm_reg_10shot_account_age_days_09_07_2026_17_06_10</t>
         </is>
       </c>
-      <c r="H13" s="21" t="n">
+      <c r="H13" s="32" t="n">
         <v>0.04791936550448601</v>
       </c>
-      <c r="I13" s="21" t="n">
+      <c r="I13" s="32" t="n">
         <v>7.243621124622016</v>
       </c>
-      <c r="J13" s="21" t="n">
+      <c r="J13" s="32" t="n">
         <v>7.127015113830566</v>
       </c>
-      <c r="K13" s="21" t="n">
+      <c r="K13" s="32" t="n">
         <v>-30.09417152404785</v>
       </c>
       <c r="L13" s="9" t="inlineStr">
@@ -2929,16 +4382,16 @@
           <t>eval_NM_to_ukr_rus_twitter_reg_10shot_account_age_days_09_07_2026_17_06_25</t>
         </is>
       </c>
-      <c r="H14" s="21" t="n">
+      <c r="H14" s="32" t="n">
         <v>-0.009068415310604738</v>
       </c>
-      <c r="I14" s="21" t="n">
+      <c r="I14" s="32" t="n">
         <v>7.44086258471682</v>
       </c>
-      <c r="J14" s="21" t="n">
+      <c r="J14" s="32" t="n">
         <v>7.313297748565674</v>
       </c>
-      <c r="K14" s="21" t="n">
+      <c r="K14" s="32" t="n">
         <v>-29.15430641174316</v>
       </c>
       <c r="L14" s="9" t="inlineStr">
@@ -2981,16 +4434,16 @@
           <t>eval_NM_to_ukr_rus_twitter_reg_10shot_followers_count_09_07_2026_17_06_26</t>
         </is>
       </c>
-      <c r="H15" s="21" t="n">
+      <c r="H15" s="32" t="n">
         <v>-0.04662848714671848</v>
       </c>
-      <c r="I15" s="21" t="n">
+      <c r="I15" s="32" t="n">
         <v>5.407601248277833</v>
       </c>
-      <c r="J15" s="21" t="n">
+      <c r="J15" s="32" t="n">
         <v>4.908641815185547</v>
       </c>
-      <c r="K15" s="21" t="n">
+      <c r="K15" s="32" t="n">
         <v>-4.749887943267822</v>
       </c>
       <c r="L15" s="9" t="inlineStr">
@@ -3033,16 +4486,16 @@
           <t>eval_NM_to_ukr_rus_twitter_reg_10shot_statuses_count_09_07_2026_17_06_26</t>
         </is>
       </c>
-      <c r="H16" s="21" t="n">
+      <c r="H16" s="32" t="n">
         <v>-0.01775905741009257</v>
       </c>
-      <c r="I16" s="21" t="n">
+      <c r="I16" s="32" t="n">
         <v>8.146453235450554</v>
       </c>
-      <c r="J16" s="21" t="n">
+      <c r="J16" s="32" t="n">
         <v>7.745946407318115</v>
       </c>
-      <c r="K16" s="21" t="n">
+      <c r="K16" s="32" t="n">
         <v>-9.51509952545166</v>
       </c>
       <c r="L16" s="9" t="inlineStr">
@@ -3085,16 +4538,16 @@
           <t>eval_CL_to_ukr_rus_twitter_reg_10shot_followers_count_09_07_2026_17_06_27</t>
         </is>
       </c>
-      <c r="H17" s="21" t="n">
+      <c r="H17" s="32" t="n">
         <v>-0.1412726350964995</v>
       </c>
-      <c r="I17" s="21" t="n">
+      <c r="I17" s="32" t="n">
         <v>5.415484000966273</v>
       </c>
-      <c r="J17" s="21" t="n">
+      <c r="J17" s="32" t="n">
         <v>4.904922962188721</v>
       </c>
-      <c r="K17" s="21" t="n">
+      <c r="K17" s="32" t="n">
         <v>-4.766663074493408</v>
       </c>
       <c r="L17" s="9" t="inlineStr">
@@ -3137,16 +4590,16 @@
           <t>eval_CL_to_ukr_rus_twitter_reg_10shot_statuses_count_09_07_2026_17_08_19</t>
         </is>
       </c>
-      <c r="H18" s="21" t="n">
+      <c r="H18" s="32" t="n">
         <v>-0.1872928742281436</v>
       </c>
-      <c r="I18" s="21" t="n">
+      <c r="I18" s="32" t="n">
         <v>8.166681510237096</v>
       </c>
-      <c r="J18" s="21" t="n">
+      <c r="J18" s="32" t="n">
         <v>7.75007963180542</v>
       </c>
-      <c r="K18" s="21" t="n">
+      <c r="K18" s="32" t="n">
         <v>-9.567384719848633</v>
       </c>
       <c r="L18" s="9" t="inlineStr">
@@ -3189,16 +4642,16 @@
           <t>eval_CL_to_ukr_rus_twitter_reg_10shot_account_age_days_09_07_2026_17_08_20</t>
         </is>
       </c>
-      <c r="H19" s="21" t="n">
+      <c r="H19" s="32" t="n">
         <v>-0.06336186652941242</v>
       </c>
-      <c r="I19" s="21" t="n">
+      <c r="I19" s="32" t="n">
         <v>7.44838424673183</v>
       </c>
-      <c r="J19" s="21" t="n">
+      <c r="J19" s="32" t="n">
         <v>7.31660795211792</v>
       </c>
-      <c r="K19" s="21" t="n">
+      <c r="K19" s="32" t="n">
         <v>-29.21529960632324</v>
       </c>
       <c r="L19" s="9" t="inlineStr">
@@ -3241,16 +4694,16 @@
           <t>eval_FP_to_ukr_rus_twitter_reg_10shot_followers_count_09_07_2026_17_08_21</t>
         </is>
       </c>
-      <c r="H20" s="21" t="n">
+      <c r="H20" s="32" t="n">
         <v>0.2751052679980367</v>
       </c>
-      <c r="I20" s="21" t="n">
+      <c r="I20" s="32" t="n">
         <v>5.171886616950228</v>
       </c>
-      <c r="J20" s="21" t="n">
+      <c r="J20" s="32" t="n">
         <v>4.665875434875488</v>
       </c>
-      <c r="K20" s="21" t="n">
+      <c r="K20" s="32" t="n">
         <v>-4.259543418884277</v>
       </c>
       <c r="L20" s="9" t="inlineStr">
@@ -3293,16 +4746,16 @@
           <t>eval_FP_to_ukr_rus_twitter_reg_10shot_statuses_count_09_07_2026_17_08_21</t>
         </is>
       </c>
-      <c r="H21" s="21" t="n">
+      <c r="H21" s="32" t="n">
         <v>0.2533726234392273</v>
       </c>
-      <c r="I21" s="21" t="n">
+      <c r="I21" s="32" t="n">
         <v>7.907792856809727</v>
       </c>
-      <c r="J21" s="21" t="n">
+      <c r="J21" s="32" t="n">
         <v>7.502818584442139</v>
       </c>
-      <c r="K21" s="21" t="n">
+      <c r="K21" s="32" t="n">
         <v>-8.908019065856934</v>
       </c>
       <c r="L21" s="9" t="inlineStr">
@@ -3345,16 +4798,16 @@
           <t>eval_FP_to_ukr_rus_twitter_reg_10shot_account_age_days_09_07_2026_17_10_15</t>
         </is>
       </c>
-      <c r="H22" s="21" t="n">
+      <c r="H22" s="32" t="n">
         <v>0.07353549289401182</v>
       </c>
-      <c r="I22" s="21" t="n">
+      <c r="I22" s="32" t="n">
         <v>7.199485008047695</v>
       </c>
-      <c r="J22" s="21" t="n">
+      <c r="J22" s="32" t="n">
         <v>7.071628093719482</v>
       </c>
-      <c r="K22" s="21" t="n">
+      <c r="K22" s="32" t="n">
         <v>-27.22965812683105</v>
       </c>
       <c r="L22" s="9" t="inlineStr">
@@ -3374,7 +4827,7 @@
           <t>ukr_rus_twitter</t>
         </is>
       </c>
-      <c r="C23" s="22" t="n">
+      <c r="C23" s="33" t="n">
         <v>10</v>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -3392,21 +4845,21 @@
           <t>test</t>
         </is>
       </c>
-      <c r="G23" s="22" t="inlineStr">
+      <c r="G23" s="33" t="inlineStr">
         <is>
           <t>eval_MIX_to_ukr_rus_twitter_reg_10shot_followers_count_09_07_2026_17_10_15</t>
         </is>
       </c>
-      <c r="H23" s="23" t="n">
+      <c r="H23" s="34" t="n">
         <v>0.178914484705714</v>
       </c>
-      <c r="I23" s="23" t="n">
+      <c r="I23" s="34" t="n">
         <v>5.184436858890582</v>
       </c>
-      <c r="J23" s="23" t="n">
+      <c r="J23" s="34" t="n">
         <v>4.684032440185547</v>
       </c>
-      <c r="K23" s="23" t="n">
+      <c r="K23" s="34" t="n">
         <v>-4.28510046005249</v>
       </c>
       <c r="L23" s="12" t="inlineStr">
@@ -3426,7 +4879,7 @@
           <t>ukr_rus_twitter</t>
         </is>
       </c>
-      <c r="C24" s="22" t="n">
+      <c r="C24" s="33" t="n">
         <v>10</v>
       </c>
       <c r="D24" s="12" t="inlineStr">
@@ -3444,21 +4897,21 @@
           <t>test</t>
         </is>
       </c>
-      <c r="G24" s="22" t="inlineStr">
+      <c r="G24" s="33" t="inlineStr">
         <is>
           <t>eval_MIX_to_ukr_rus_twitter_reg_10shot_account_age_days_09_07_2026_17_10_19</t>
         </is>
       </c>
-      <c r="H24" s="23" t="n">
+      <c r="H24" s="34" t="n">
         <v>0.07703031346775366</v>
       </c>
-      <c r="I24" s="23" t="n">
+      <c r="I24" s="34" t="n">
         <v>7.196615260642798</v>
       </c>
-      <c r="J24" s="23" t="n">
+      <c r="J24" s="34" t="n">
         <v>7.068069458007812</v>
       </c>
-      <c r="K24" s="23" t="n">
+      <c r="K24" s="34" t="n">
         <v>-27.20715713500977</v>
       </c>
       <c r="L24" s="12" t="inlineStr">
@@ -3478,7 +4931,7 @@
           <t>ukr_rus_twitter</t>
         </is>
       </c>
-      <c r="C25" s="22" t="n">
+      <c r="C25" s="33" t="n">
         <v>10</v>
       </c>
       <c r="D25" s="12" t="inlineStr">
@@ -3496,21 +4949,21 @@
           <t>test</t>
         </is>
       </c>
-      <c r="G25" s="22" t="inlineStr">
+      <c r="G25" s="33" t="inlineStr">
         <is>
           <t>eval_MIX_to_ukr_rus_twitter_reg_10shot_statuses_count_09_07_2026_17_10_19</t>
         </is>
       </c>
-      <c r="H25" s="23" t="n">
+      <c r="H25" s="34" t="n">
         <v>0.1401208974693679</v>
       </c>
-      <c r="I25" s="23" t="n">
+      <c r="I25" s="34" t="n">
         <v>7.902268202416312</v>
       </c>
-      <c r="J25" s="23" t="n">
+      <c r="J25" s="34" t="n">
         <v>7.49895191192627</v>
       </c>
-      <c r="K25" s="23" t="n">
+      <c r="K25" s="34" t="n">
         <v>-8.894180297851562</v>
       </c>
       <c r="L25" s="12" t="inlineStr">
@@ -3553,16 +5006,16 @@
           <t>eval_NM_to_covid19_twitter_reg_10shot_statuses_count_09_07_2026_17_12_10</t>
         </is>
       </c>
-      <c r="H26" s="21" t="n">
+      <c r="H26" s="32" t="n">
         <v>-0.02848686181695186</v>
       </c>
-      <c r="I26" s="21" t="n">
+      <c r="I26" s="32" t="n">
         <v>8.191415098200991</v>
       </c>
-      <c r="J26" s="21" t="n">
+      <c r="J26" s="32" t="n">
         <v>7.889354228973389</v>
       </c>
-      <c r="K26" s="21" t="n">
+      <c r="K26" s="32" t="n">
         <v>-13.00656127929688</v>
       </c>
       <c r="L26" s="9" t="inlineStr">
@@ -3605,16 +5058,16 @@
           <t>eval_NM_to_covid19_twitter_reg_10shot_followers_count_09_07_2026_17_12_10</t>
         </is>
       </c>
-      <c r="H27" s="21" t="n">
+      <c r="H27" s="32" t="n">
         <v>-0.0765577187841977</v>
       </c>
-      <c r="I27" s="21" t="n">
+      <c r="I27" s="32" t="n">
         <v>5.556185964208908</v>
       </c>
-      <c r="J27" s="21" t="n">
+      <c r="J27" s="32" t="n">
         <v>5.172481060028076</v>
       </c>
-      <c r="K27" s="21" t="n">
+      <c r="K27" s="32" t="n">
         <v>-6.668301105499268</v>
       </c>
       <c r="L27" s="9" t="inlineStr">
@@ -3657,16 +5110,16 @@
           <t>eval_NM_to_covid19_twitter_reg_10shot_account_age_days_09_07_2026_17_12_10</t>
         </is>
       </c>
-      <c r="H28" s="21" t="n">
+      <c r="H28" s="32" t="n">
         <v>0.04410056145581293</v>
       </c>
-      <c r="I28" s="21" t="n">
+      <c r="I28" s="32" t="n">
         <v>7.460839076166901</v>
       </c>
-      <c r="J28" s="21" t="n">
+      <c r="J28" s="32" t="n">
         <v>7.375690937042236</v>
       </c>
-      <c r="K28" s="21" t="n">
+      <c r="K28" s="32" t="n">
         <v>-44.13318252563477</v>
       </c>
       <c r="L28" s="9" t="inlineStr">
@@ -3709,16 +5162,16 @@
           <t>eval_CL_to_covid19_twitter_reg_10shot_followers_count_09_07_2026_17_12_13</t>
         </is>
       </c>
-      <c r="H29" s="21" t="n">
+      <c r="H29" s="32" t="n">
         <v>-0.1685501218130046</v>
       </c>
-      <c r="I29" s="21" t="n">
+      <c r="I29" s="32" t="n">
         <v>5.59294011737066</v>
       </c>
-      <c r="J29" s="21" t="n">
+      <c r="J29" s="32" t="n">
         <v>5.199687004089355</v>
       </c>
-      <c r="K29" s="21" t="n">
+      <c r="K29" s="32" t="n">
         <v>-6.770088195800781</v>
       </c>
       <c r="L29" s="9" t="inlineStr">
@@ -3761,16 +5214,16 @@
           <t>eval_CL_to_covid19_twitter_reg_10shot_statuses_count_09_07_2026_17_16_13</t>
         </is>
       </c>
-      <c r="H30" s="21" t="n">
+      <c r="H30" s="32" t="n">
         <v>-0.2157195553808251</v>
       </c>
-      <c r="I30" s="21" t="n">
+      <c r="I30" s="32" t="n">
         <v>8.245818494488159</v>
       </c>
-      <c r="J30" s="21" t="n">
+      <c r="J30" s="32" t="n">
         <v>7.929580688476562</v>
       </c>
-      <c r="K30" s="21" t="n">
+      <c r="K30" s="32" t="n">
         <v>-13.19322967529297</v>
       </c>
       <c r="L30" s="9" t="inlineStr">
@@ -3813,16 +5266,16 @@
           <t>eval_CL_to_covid19_twitter_reg_10shot_account_age_days_09_07_2026_17_16_13</t>
         </is>
       </c>
-      <c r="H31" s="21" t="n">
+      <c r="H31" s="32" t="n">
         <v>-0.0885545605857191</v>
       </c>
-      <c r="I31" s="21" t="n">
+      <c r="I31" s="32" t="n">
         <v>7.505862932603892</v>
       </c>
-      <c r="J31" s="21" t="n">
+      <c r="J31" s="32" t="n">
         <v>7.415299415588379</v>
       </c>
-      <c r="K31" s="21" t="n">
+      <c r="K31" s="32" t="n">
         <v>-44.67955780029297</v>
       </c>
       <c r="L31" s="9" t="inlineStr">
@@ -3865,16 +5318,16 @@
           <t>eval_FP_to_covid19_twitter_reg_10shot_followers_count_09_07_2026_17_16_14</t>
         </is>
       </c>
-      <c r="H32" s="21" t="n">
+      <c r="H32" s="32" t="n">
         <v>0.2403043542668442</v>
       </c>
-      <c r="I32" s="21" t="n">
+      <c r="I32" s="32" t="n">
         <v>5.325212773473345</v>
       </c>
-      <c r="J32" s="21" t="n">
+      <c r="J32" s="32" t="n">
         <v>4.939977645874023</v>
       </c>
-      <c r="K32" s="21" t="n">
+      <c r="K32" s="32" t="n">
         <v>-6.044003009796143</v>
       </c>
       <c r="L32" s="9" t="inlineStr">
@@ -3917,16 +5370,16 @@
           <t>eval_FP_to_covid19_twitter_reg_10shot_statuses_count_09_07_2026_17_16_14</t>
         </is>
       </c>
-      <c r="H33" s="21" t="n">
+      <c r="H33" s="32" t="n">
         <v>0.2305739948085812</v>
       </c>
-      <c r="I33" s="21" t="n">
+      <c r="I33" s="32" t="n">
         <v>7.961909930105177</v>
       </c>
-      <c r="J33" s="21" t="n">
+      <c r="J33" s="32" t="n">
         <v>7.658311367034912</v>
       </c>
-      <c r="K33" s="21" t="n">
+      <c r="K33" s="32" t="n">
         <v>-12.23269176483154</v>
       </c>
       <c r="L33" s="9" t="inlineStr">
@@ -3969,16 +5422,16 @@
           <t>eval_FP_to_covid19_twitter_reg_10shot_account_age_days_09_07_2026_17_20_28</t>
         </is>
       </c>
-      <c r="H34" s="21" t="n">
+      <c r="H34" s="32" t="n">
         <v>0.05878688358840294</v>
       </c>
-      <c r="I34" s="21" t="n">
+      <c r="I34" s="32" t="n">
         <v>7.231221312892131</v>
       </c>
-      <c r="J34" s="21" t="n">
+      <c r="J34" s="32" t="n">
         <v>7.145621776580811</v>
       </c>
-      <c r="K34" s="21" t="n">
+      <c r="K34" s="32" t="n">
         <v>-41.39786148071289</v>
       </c>
       <c r="L34" s="9" t="inlineStr">
@@ -3998,7 +5451,7 @@
           <t>covid19_twitter</t>
         </is>
       </c>
-      <c r="C35" s="22" t="n">
+      <c r="C35" s="33" t="n">
         <v>10</v>
       </c>
       <c r="D35" s="12" t="inlineStr">
@@ -4016,21 +5469,21 @@
           <t>test</t>
         </is>
       </c>
-      <c r="G35" s="22" t="inlineStr">
+      <c r="G35" s="33" t="inlineStr">
         <is>
           <t>eval_MIX_to_covid19_twitter_reg_10shot_followers_count_09_07_2026_17_20_34</t>
         </is>
       </c>
-      <c r="H35" s="23" t="n">
+      <c r="H35" s="34" t="n">
         <v>0.1607689020878813</v>
       </c>
-      <c r="I35" s="23" t="n">
+      <c r="I35" s="34" t="n">
         <v>5.331860795981971</v>
       </c>
-      <c r="J35" s="23" t="n">
+      <c r="J35" s="34" t="n">
         <v>4.950477123260498</v>
       </c>
-      <c r="K35" s="23" t="n">
+      <c r="K35" s="34" t="n">
         <v>-6.061601638793945</v>
       </c>
       <c r="L35" s="12" t="inlineStr">
@@ -4050,7 +5503,7 @@
           <t>covid19_twitter</t>
         </is>
       </c>
-      <c r="C36" s="22" t="n">
+      <c r="C36" s="33" t="n">
         <v>10</v>
       </c>
       <c r="D36" s="12" t="inlineStr">
@@ -4068,21 +5521,21 @@
           <t>test</t>
         </is>
       </c>
-      <c r="G36" s="22" t="inlineStr">
+      <c r="G36" s="33" t="inlineStr">
         <is>
           <t>eval_MIX_to_covid19_twitter_reg_10shot_account_age_days_09_07_2026_17_20_35</t>
         </is>
       </c>
-      <c r="H36" s="23" t="n">
+      <c r="H36" s="34" t="n">
         <v>0.07518974943342481</v>
       </c>
-      <c r="I36" s="23" t="n">
+      <c r="I36" s="34" t="n">
         <v>7.222926925447974</v>
       </c>
-      <c r="J36" s="23" t="n">
+      <c r="J36" s="34" t="n">
         <v>7.136369705200195</v>
       </c>
-      <c r="K36" s="23" t="n">
+      <c r="K36" s="34" t="n">
         <v>-41.30065155029297</v>
       </c>
       <c r="L36" s="12" t="inlineStr">
@@ -4102,7 +5555,7 @@
           <t>covid19_twitter</t>
         </is>
       </c>
-      <c r="C37" s="22" t="n">
+      <c r="C37" s="33" t="n">
         <v>10</v>
       </c>
       <c r="D37" s="12" t="inlineStr">
@@ -4120,21 +5573,21 @@
           <t>test</t>
         </is>
       </c>
-      <c r="G37" s="22" t="inlineStr">
+      <c r="G37" s="33" t="inlineStr">
         <is>
           <t>eval_MIX_to_covid19_twitter_reg_10shot_statuses_count_09_07_2026_17_20_35</t>
         </is>
       </c>
-      <c r="H37" s="23" t="n">
+      <c r="H37" s="34" t="n">
         <v>0.1202913704609749</v>
       </c>
-      <c r="I37" s="23" t="n">
+      <c r="I37" s="34" t="n">
         <v>7.949625200757551</v>
       </c>
-      <c r="J37" s="23" t="n">
+      <c r="J37" s="34" t="n">
         <v>7.647272109985352</v>
       </c>
-      <c r="K37" s="23" t="n">
+      <c r="K37" s="34" t="n">
         <v>-12.1918888092041</v>
       </c>
       <c r="L37" s="12" t="inlineStr">
@@ -4177,16 +5630,16 @@
           <t>eval_NM_to_twibot20_reg_10shot_statuses_count_09_07_2026_17_25_27</t>
         </is>
       </c>
-      <c r="H38" s="21" t="n">
+      <c r="H38" s="32" t="n">
         <v>0.06259008073215844</v>
       </c>
-      <c r="I38" s="21" t="n">
+      <c r="I38" s="32" t="n">
         <v>8.449133870354977</v>
       </c>
-      <c r="J38" s="21" t="n">
+      <c r="J38" s="32" t="n">
         <v>8.105243682861328</v>
       </c>
-      <c r="K38" s="21" t="n">
+      <c r="K38" s="32" t="n">
         <v>-11.48660087585449</v>
       </c>
       <c r="L38" s="9" t="inlineStr">
@@ -4229,16 +5682,16 @@
           <t>eval_NM_to_twibot20_reg_10shot_followers_count_09_07_2026_17_25_27</t>
         </is>
       </c>
-      <c r="H39" s="21" t="n">
+      <c r="H39" s="32" t="n">
         <v>0.1413114953751201</v>
       </c>
-      <c r="I39" s="21" t="n">
+      <c r="I39" s="32" t="n">
         <v>8.317230026133531</v>
       </c>
-      <c r="J39" s="21" t="n">
+      <c r="J39" s="32" t="n">
         <v>7.75342321395874</v>
       </c>
-      <c r="K39" s="21" t="n">
+      <c r="K39" s="32" t="n">
         <v>-6.533519744873047</v>
       </c>
       <c r="L39" s="9" t="inlineStr">
@@ -4281,16 +5734,16 @@
           <t>eval_NM_to_twibot20_reg_10shot_account_age_days_09_07_2026_17_25_28</t>
         </is>
       </c>
-      <c r="H40" s="21" t="n">
+      <c r="H40" s="32" t="n">
         <v>0.05647117118237376</v>
       </c>
-      <c r="I40" s="21" t="n">
+      <c r="I40" s="32" t="n">
         <v>7.772332040978731</v>
       </c>
-      <c r="J40" s="21" t="n">
+      <c r="J40" s="32" t="n">
         <v>7.68785285949707</v>
       </c>
-      <c r="K40" s="21" t="n">
+      <c r="K40" s="32" t="n">
         <v>-45.90118408203125</v>
       </c>
       <c r="L40" s="9" t="inlineStr">
@@ -4333,16 +5786,16 @@
           <t>eval_CL_to_twibot20_reg_10shot_followers_count_09_07_2026_17_25_28</t>
         </is>
       </c>
-      <c r="H41" s="21" t="n">
+      <c r="H41" s="32" t="n">
         <v>-0.06590133623730586</v>
       </c>
-      <c r="I41" s="21" t="n">
+      <c r="I41" s="32" t="n">
         <v>8.385390483428324</v>
       </c>
-      <c r="J41" s="21" t="n">
+      <c r="J41" s="32" t="n">
         <v>7.81448221206665</v>
       </c>
-      <c r="K41" s="21" t="n">
+      <c r="K41" s="32" t="n">
         <v>-6.657500743865967</v>
       </c>
       <c r="L41" s="9" t="inlineStr">
@@ -4385,16 +5838,16 @@
           <t>eval_CL_to_twibot20_reg_10shot_statuses_count_09_07_2026_17_25_41</t>
         </is>
       </c>
-      <c r="H42" s="21" t="n">
+      <c r="H42" s="32" t="n">
         <v>-0.05816875177586175</v>
       </c>
-      <c r="I42" s="21" t="n">
+      <c r="I42" s="32" t="n">
         <v>8.52563604851499</v>
       </c>
-      <c r="J42" s="21" t="n">
+      <c r="J42" s="32" t="n">
         <v>8.169377326965332</v>
       </c>
-      <c r="K42" s="21" t="n">
+      <c r="K42" s="32" t="n">
         <v>-11.71374225616455</v>
       </c>
       <c r="L42" s="9" t="inlineStr">
@@ -4437,16 +5890,16 @@
           <t>eval_CL_to_twibot20_reg_10shot_account_age_days_09_07_2026_17_25_41</t>
         </is>
       </c>
-      <c r="H43" s="21" t="n">
+      <c r="H43" s="32" t="n">
         <v>-0.07570675745125917</v>
       </c>
-      <c r="I43" s="21" t="n">
+      <c r="I43" s="32" t="n">
         <v>7.846535237566642</v>
       </c>
-      <c r="J43" s="21" t="n">
+      <c r="J43" s="32" t="n">
         <v>7.753562927246094</v>
       </c>
-      <c r="K43" s="21" t="n">
+      <c r="K43" s="32" t="n">
         <v>-46.80099868774414</v>
       </c>
       <c r="L43" s="9" t="inlineStr">
@@ -4489,16 +5942,16 @@
           <t>eval_FP_to_twibot20_reg_10shot_statuses_count_09_07_2026_17_25_42</t>
         </is>
       </c>
-      <c r="H44" s="21" t="n">
+      <c r="H44" s="32" t="n">
         <v>0.1515542906059071</v>
       </c>
-      <c r="I44" s="21" t="n">
+      <c r="I44" s="32" t="n">
         <v>8.228838512460927</v>
       </c>
-      <c r="J44" s="21" t="n">
+      <c r="J44" s="32" t="n">
         <v>7.876864433288574</v>
       </c>
-      <c r="K44" s="21" t="n">
+      <c r="K44" s="32" t="n">
         <v>-10.84395885467529</v>
       </c>
       <c r="L44" s="9" t="inlineStr">
@@ -4541,16 +5994,16 @@
           <t>eval_FP_to_twibot20_reg_10shot_followers_count_09_07_2026_17_25_42</t>
         </is>
       </c>
-      <c r="H45" s="21" t="n">
+      <c r="H45" s="32" t="n">
         <v>0.1044004024775087</v>
       </c>
-      <c r="I45" s="21" t="n">
+      <c r="I45" s="32" t="n">
         <v>8.106635834652009</v>
       </c>
-      <c r="J45" s="21" t="n">
+      <c r="J45" s="32" t="n">
         <v>7.523114681243896</v>
       </c>
-      <c r="K45" s="21" t="n">
+      <c r="K45" s="32" t="n">
         <v>-6.156847953796387</v>
       </c>
       <c r="L45" s="9" t="inlineStr">
@@ -4593,16 +6046,16 @@
           <t>eval_FP_to_twibot20_reg_10shot_account_age_days_09_07_2026_17_25_55</t>
         </is>
       </c>
-      <c r="H46" s="21" t="n">
+      <c r="H46" s="32" t="n">
         <v>0.05774584604707877</v>
       </c>
-      <c r="I46" s="21" t="n">
+      <c r="I46" s="32" t="n">
         <v>7.546795641242951</v>
       </c>
-      <c r="J46" s="21" t="n">
+      <c r="J46" s="32" t="n">
         <v>7.461183071136475</v>
       </c>
-      <c r="K46" s="21" t="n">
+      <c r="K46" s="32" t="n">
         <v>-43.21873474121094</v>
       </c>
       <c r="L46" s="9" t="inlineStr">
@@ -4622,7 +6075,7 @@
           <t>twibot20</t>
         </is>
       </c>
-      <c r="C47" s="22" t="n">
+      <c r="C47" s="33" t="n">
         <v>10</v>
       </c>
       <c r="D47" s="12" t="inlineStr">
@@ -4640,21 +6093,21 @@
           <t>test</t>
         </is>
       </c>
-      <c r="G47" s="22" t="inlineStr">
+      <c r="G47" s="33" t="inlineStr">
         <is>
           <t>eval_MIX_to_twibot20_reg_10shot_statuses_count_09_07_2026_17_25_56</t>
         </is>
       </c>
-      <c r="H47" s="23" t="n">
+      <c r="H47" s="34" t="n">
         <v>0.02228732147364963</v>
       </c>
-      <c r="I47" s="23" t="n">
+      <c r="I47" s="34" t="n">
         <v>8.151193973633603</v>
       </c>
-      <c r="J47" s="23" t="n">
+      <c r="J47" s="34" t="n">
         <v>7.793371200561523</v>
       </c>
-      <c r="K47" s="23" t="n">
+      <c r="K47" s="34" t="n">
         <v>-10.62150287628174</v>
       </c>
       <c r="L47" s="12" t="inlineStr">
@@ -4674,7 +6127,7 @@
           <t>twibot20</t>
         </is>
       </c>
-      <c r="C48" s="22" t="n">
+      <c r="C48" s="33" t="n">
         <v>10</v>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -4692,21 +6145,21 @@
           <t>test</t>
         </is>
       </c>
-      <c r="G48" s="22" t="inlineStr">
+      <c r="G48" s="33" t="inlineStr">
         <is>
           <t>eval_MIX_to_twibot20_reg_10shot_followers_count_09_07_2026_17_25_56</t>
         </is>
       </c>
-      <c r="H48" s="23" t="n">
+      <c r="H48" s="34" t="n">
         <v>-0.1053002475786942</v>
       </c>
-      <c r="I48" s="23" t="n">
+      <c r="I48" s="34" t="n">
         <v>8.047293109586699</v>
       </c>
-      <c r="J48" s="23" t="n">
+      <c r="J48" s="34" t="n">
         <v>7.443381309509277</v>
       </c>
-      <c r="K48" s="23" t="n">
+      <c r="K48" s="34" t="n">
         <v>-6.052451610565186</v>
       </c>
       <c r="L48" s="12" t="inlineStr">
@@ -4726,7 +6179,7 @@
           <t>twibot20</t>
         </is>
       </c>
-      <c r="C49" s="22" t="n">
+      <c r="C49" s="33" t="n">
         <v>10</v>
       </c>
       <c r="D49" s="12" t="inlineStr">
@@ -4744,776 +6197,26 @@
           <t>test</t>
         </is>
       </c>
-      <c r="G49" s="22" t="inlineStr">
+      <c r="G49" s="33" t="inlineStr">
         <is>
           <t>eval_MIX_to_twibot20_reg_10shot_account_age_days_09_07_2026_17_25_56</t>
         </is>
       </c>
-      <c r="H49" s="23" t="n">
+      <c r="H49" s="34" t="n">
         <v>-0.03517145990771501</v>
       </c>
-      <c r="I49" s="23" t="n">
+      <c r="I49" s="34" t="n">
         <v>7.464907882949912</v>
       </c>
-      <c r="J49" s="23" t="n">
+      <c r="J49" s="34" t="n">
         <v>7.375756740570068</v>
       </c>
-      <c r="K49" s="23" t="n">
+      <c r="K49" s="34" t="n">
         <v>-42.26433181762695</v>
       </c>
       <c r="L49" s="12" t="inlineStr">
         <is>
           <t>55.724849700927734</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>dataset</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>shots</t>
-        </is>
-      </c>
-      <c r="D1" s="6" t="inlineStr">
-        <is>
-          <t>target</t>
-        </is>
-      </c>
-      <c r="E1" s="6" t="inlineStr">
-        <is>
-          <t>task</t>
-        </is>
-      </c>
-      <c r="F1" s="6" t="inlineStr">
-        <is>
-          <t>split</t>
-        </is>
-      </c>
-      <c r="G1" s="6" t="inlineStr">
-        <is>
-          <t>run</t>
-        </is>
-      </c>
-      <c r="H1" s="6" t="inlineStr">
-        <is>
-          <t>roc_auc</t>
-        </is>
-      </c>
-      <c r="I1" s="6" t="inlineStr">
-        <is>
-          <t>accuracy</t>
-        </is>
-      </c>
-      <c r="J1" s="6" t="inlineStr">
-        <is>
-          <t>f1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B2" s="9" t="inlineStr">
-        <is>
-          <t>midterm</t>
-        </is>
-      </c>
-      <c r="C2" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="9" t="inlineStr"/>
-      <c r="E2" s="9" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F2" s="9" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G2" s="13" t="inlineStr">
-        <is>
-          <t>eval_CL_to_midterm_slp_0shot_09_07_2026_17_28_00</t>
-        </is>
-      </c>
-      <c r="H2" s="21" t="n">
-        <v>0.416752375</v>
-      </c>
-      <c r="I2" s="21" t="n">
-        <v>0.498</v>
-      </c>
-      <c r="J2" s="9" t="inlineStr">
-        <is>
-          <t>0.664886515353805</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>FP</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>midterm</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="9" t="inlineStr"/>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G3" s="13" t="inlineStr">
-        <is>
-          <t>eval_FP_to_midterm_slp_0shot_09_07_2026_17_28_00</t>
-        </is>
-      </c>
-      <c r="H3" s="21" t="n">
-        <v>0.433355</v>
-      </c>
-      <c r="I3" s="21" t="n">
-        <v>0.5465</v>
-      </c>
-      <c r="J3" s="9" t="inlineStr">
-        <is>
-          <t>0.6625744047619048</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>NM</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>midterm</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="9" t="inlineStr"/>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G4" s="13" t="inlineStr">
-        <is>
-          <t>eval_NM_to_midterm_slp_0shot_09_07_2026_17_28_00</t>
-        </is>
-      </c>
-      <c r="H4" s="21" t="n">
-        <v>0.48701</v>
-      </c>
-      <c r="I4" s="21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J4" s="9" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>MIX</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>midterm</t>
-        </is>
-      </c>
-      <c r="C5" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="12" t="inlineStr"/>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G5" s="22" t="inlineStr">
-        <is>
-          <t>eval_MIX_to_midterm_slp_0shot_09_07_2026_17_28_01</t>
-        </is>
-      </c>
-      <c r="H5" s="23" t="n">
-        <v>0.676129875</v>
-      </c>
-      <c r="I5" s="23" t="n">
-        <v>0.64225</v>
-      </c>
-      <c r="J5" s="12" t="inlineStr">
-        <is>
-          <t>0.5343312723722746</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>ukr_rus_twitter</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr"/>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G6" s="13" t="inlineStr">
-        <is>
-          <t>eval_CL_to_ukr_rus_twitter_slp_0shot_09_07_2026_17_28_20</t>
-        </is>
-      </c>
-      <c r="H6" s="21" t="n">
-        <v>0.2875115</v>
-      </c>
-      <c r="I6" s="21" t="n">
-        <v>0.4995</v>
-      </c>
-      <c r="J6" s="9" t="inlineStr">
-        <is>
-          <t>0.6662220740246749</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>NM</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>ukr_rus_twitter</t>
-        </is>
-      </c>
-      <c r="C7" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="9" t="inlineStr"/>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G7" s="13" t="inlineStr">
-        <is>
-          <t>eval_NM_to_ukr_rus_twitter_slp_0shot_09_07_2026_17_28_20</t>
-        </is>
-      </c>
-      <c r="H7" s="21" t="n">
-        <v>0.48371125</v>
-      </c>
-      <c r="I7" s="21" t="n">
-        <v>0.49975</v>
-      </c>
-      <c r="J7" s="9" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>FP</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>ukr_rus_twitter</t>
-        </is>
-      </c>
-      <c r="C8" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="9" t="inlineStr"/>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G8" s="13" t="inlineStr">
-        <is>
-          <t>eval_FP_to_ukr_rus_twitter_slp_0shot_09_07_2026_17_28_21</t>
-        </is>
-      </c>
-      <c r="H8" s="21" t="n">
-        <v>0.53384625</v>
-      </c>
-      <c r="I8" s="21" t="n">
-        <v>0.55925</v>
-      </c>
-      <c r="J8" s="9" t="inlineStr">
-        <is>
-          <t>0.6713886300093197</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>MIX</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>ukr_rus_twitter</t>
-        </is>
-      </c>
-      <c r="C9" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="12" t="inlineStr"/>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G9" s="22" t="inlineStr">
-        <is>
-          <t>eval_MIX_to_ukr_rus_twitter_slp_0shot_09_07_2026_17_28_21</t>
-        </is>
-      </c>
-      <c r="H9" s="23" t="n">
-        <v>0.8612627499999999</v>
-      </c>
-      <c r="I9" s="23" t="n">
-        <v>0.779</v>
-      </c>
-      <c r="J9" s="12" t="inlineStr">
-        <is>
-          <t>0.7390791027154664</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>covid19_twitter</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr"/>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>eval_CL_to_covid19_twitter_slp_0shot_09_07_2026_17_34_22</t>
-        </is>
-      </c>
-      <c r="H10" s="21" t="n">
-        <v>0.366347875</v>
-      </c>
-      <c r="I10" s="21" t="n">
-        <v>0.49975</v>
-      </c>
-      <c r="J10" s="9" t="inlineStr">
-        <is>
-          <t>0.6661104622059069</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>FP</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>covid19_twitter</t>
-        </is>
-      </c>
-      <c r="C11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="9" t="inlineStr"/>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G11" s="13" t="inlineStr">
-        <is>
-          <t>eval_FP_to_covid19_twitter_slp_0shot_09_07_2026_17_34_22</t>
-        </is>
-      </c>
-      <c r="H11" s="21" t="n">
-        <v>0.4486818750000001</v>
-      </c>
-      <c r="I11" s="21" t="n">
-        <v>0.52425</v>
-      </c>
-      <c r="J11" s="9" t="inlineStr">
-        <is>
-          <t>0.6356500095730423</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>NM</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>covid19_twitter</t>
-        </is>
-      </c>
-      <c r="C12" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr"/>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>eval_NM_to_covid19_twitter_slp_0shot_09_07_2026_17_34_22</t>
-        </is>
-      </c>
-      <c r="H12" s="21" t="n">
-        <v>0.40565375</v>
-      </c>
-      <c r="I12" s="21" t="n">
-        <v>0.4995</v>
-      </c>
-      <c r="J12" s="9" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>MIX</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>covid19_twitter</t>
-        </is>
-      </c>
-      <c r="C13" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="12" t="inlineStr"/>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G13" s="22" t="inlineStr">
-        <is>
-          <t>eval_MIX_to_covid19_twitter_slp_0shot_09_07_2026_17_34_25</t>
-        </is>
-      </c>
-      <c r="H13" s="23" t="n">
-        <v>0.75508</v>
-      </c>
-      <c r="I13" s="23" t="n">
-        <v>0.6765</v>
-      </c>
-      <c r="J13" s="12" t="inlineStr">
-        <is>
-          <t>0.5790500975927131</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>NM</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>twibot20</t>
-        </is>
-      </c>
-      <c r="C14" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="9" t="inlineStr"/>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G14" s="13" t="inlineStr">
-        <is>
-          <t>eval_NM_to_twibot20_slp_0shot_09_07_2026_17_38_14</t>
-        </is>
-      </c>
-      <c r="H14" s="21" t="n">
-        <v>0.49065475</v>
-      </c>
-      <c r="I14" s="21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J14" s="9" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>twibot20</t>
-        </is>
-      </c>
-      <c r="C15" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr"/>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G15" s="13" t="inlineStr">
-        <is>
-          <t>eval_CL_to_twibot20_slp_0shot_09_07_2026_17_38_17</t>
-        </is>
-      </c>
-      <c r="H15" s="21" t="n">
-        <v>0.2592245</v>
-      </c>
-      <c r="I15" s="21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J15" s="9" t="inlineStr">
-        <is>
-          <t>0.6666666666666666</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>FP</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>twibot20</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr"/>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G16" s="13" t="inlineStr">
-        <is>
-          <t>eval_FP_to_twibot20_slp_0shot_09_07_2026_17_38_17</t>
-        </is>
-      </c>
-      <c r="H16" s="21" t="n">
-        <v>0.381107125</v>
-      </c>
-      <c r="I16" s="21" t="n">
-        <v>0.5135</v>
-      </c>
-      <c r="J16" s="9" t="inlineStr">
-        <is>
-          <t>0.6497480201583873</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>MIX</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>twibot20</t>
-        </is>
-      </c>
-      <c r="C17" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="12" t="inlineStr"/>
-      <c r="E17" s="12" t="inlineStr">
-        <is>
-          <t>static_link_prediction</t>
-        </is>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="G17" s="22" t="inlineStr">
-        <is>
-          <t>eval_MIX_to_twibot20_slp_0shot_09_07_2026_17_38_17</t>
-        </is>
-      </c>
-      <c r="H17" s="23" t="n">
-        <v>0.74460025</v>
-      </c>
-      <c r="I17" s="23" t="n">
-        <v>0.66475</v>
-      </c>
-      <c r="J17" s="12" t="inlineStr">
-        <is>
-          <t>0.566159818828858</t>
         </is>
       </c>
     </row>

</xml_diff>